<commit_message>
feat(fpa-engine): complete architectural cleanup, 4Q/8Q forecasting engine, historical analytics, audit trail, and unified PDF reporters
</commit_message>
<xml_diff>
--- a/Data/True_data/current_data/balance_sheet.xlsx
+++ b/Data/True_data/current_data/balance_sheet.xlsx
@@ -471,7 +471,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -491,7 +490,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>508.22</v>
+        <v>570.8</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +500,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>264.4</v>
+        <v>201.7</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +510,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>98.25</v>
+        <v>90.47</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +520,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>43.98</v>
+        <v>36.53</v>
       </c>
     </row>
     <row r="10">
@@ -531,7 +530,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>914.85</v>
+        <v>899.5</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +540,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>368.89</v>
+        <v>279.78</v>
       </c>
     </row>
     <row r="12">
@@ -551,7 +550,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>85.88</v>
+        <v>64.16</v>
       </c>
     </row>
     <row r="13">
@@ -561,7 +560,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>1369.61</v>
+        <v>1243.43</v>
       </c>
     </row>
     <row r="14">
@@ -571,7 +570,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>87.53</v>
+        <v>62.98</v>
       </c>
     </row>
     <row r="15">
@@ -581,7 +580,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>76.45999999999999</v>
+        <v>205.72</v>
       </c>
     </row>
     <row r="16">
@@ -591,7 +590,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>36.37</v>
+        <v>50.98</v>
       </c>
     </row>
     <row r="17">
@@ -601,7 +600,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>66.04000000000001</v>
+        <v>52.56</v>
       </c>
     </row>
     <row r="18">
@@ -611,7 +610,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>266.4</v>
+        <v>372.24</v>
       </c>
     </row>
     <row r="19">
@@ -621,7 +620,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>325.79</v>
+        <v>284.71</v>
       </c>
     </row>
     <row r="20">
@@ -631,7 +630,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>592.1900000000001</v>
+        <v>656.95</v>
       </c>
     </row>
     <row r="21">
@@ -641,7 +640,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>102.46</v>
+        <v>131.34</v>
       </c>
     </row>
     <row r="22">
@@ -651,7 +650,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>248.24</v>
+        <v>164.32</v>
       </c>
     </row>
     <row r="23">
@@ -661,7 +660,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>426.73</v>
+        <v>290.81</v>
       </c>
     </row>
     <row r="24">
@@ -671,7 +670,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>777.4299999999999</v>
+        <v>586.48</v>
       </c>
     </row>
     <row r="25">
@@ -681,7 +680,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1369.62</v>
+        <v>1243.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>